<commit_message>
Add English version of the Excel data matrix and improve print layout
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MD47aVtD3AvwE7o7W6NRea
</commit_message>
<xml_diff>
--- a/exports/BOMAG_Compare_Hub_Matriz_Datos.xlsx
+++ b/exports/BOMAG_Compare_Hub_Matriz_Datos.xlsx
@@ -17917,16 +17917,16 @@
     </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C39:AX39" type="list">
-      <formula1>"SÍ,NO"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5" type="list">
       <formula1>"Roca,Grava,Suelo mixto,Arcilla"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N5" type="list">
       <formula1>IDS_SDR</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C39:AX39" type="list">
+      <formula1>"SÍ,NO"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C40:AX40" type="list">
@@ -17940,7 +17940,7 @@
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.5"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="6" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter>&amp;LBOMAG Compare Hub&amp;R&amp;P / &amp;N</oddFooter>

</xml_diff>